<commit_message>
Added several extensions and resource types
</commit_message>
<xml_diff>
--- a/314e-ig/output/StructureDefinition-datetime-314e.xlsx
+++ b/314e-ig/output/StructureDefinition-datetime-314e.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-05-26T19:54:55+05:30</t>
+    <t>2026-06-10T16:33:40+05:30</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -86,7 +86,7 @@
 If only a smaller degree of precision is usable
 (for example, only the date portion is known),
 the following extension SHALL be used:
-http://314e.com/fhir/StructureDefinition/datetime-precision-314e
+http://314e.com/fhir/StructureDefinition/datetime-precision
 If all or part of the usable date/time value is approximate rather than exact,
 the following extension SHALL be used:
 https://hl7.org.au/fhir/StructureDefinition/date-accuracy-indicator</t>
@@ -315,7 +315,7 @@
     <t>timePrecision</t>
   </si>
   <si>
-    <t xml:space="preserve">Extension {http://314e.com/fhir/StructureDefinition/datetime-precision-314e}
+    <t xml:space="preserve">Extension {http://314e.com/fhir/StructureDefinition/datetime-precision}
 </t>
   </si>
   <si>
@@ -342,7 +342,7 @@
     <t>accuracyIndicator</t>
   </si>
   <si>
-    <t xml:space="preserve">Extension {http://314e.com/fhir/StructureDefinition/datetime-accuracy-314e}
+    <t xml:space="preserve">Extension {http://314e.com/fhir/StructureDefinition/datetime-accuracy}
 </t>
   </si>
   <si>
@@ -679,7 +679,7 @@
     <col min="8" max="8" width="13.1171875" customWidth="true" bestFit="true"/>
     <col min="9" max="9" width="10.75390625" customWidth="true" bestFit="true"/>
     <col min="10" max="10" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="11" max="11" width="64.0625" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" width="59.4765625" customWidth="true" bestFit="true"/>
     <col min="12" max="12" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="13" max="13" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="14" max="14" width="100.703125" customWidth="true" bestFit="true"/>

</xml_diff>